<commit_message>
Implement parser for a list of objects having only single cell values
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/SampleDataFile.xlsx
+++ b/src/test/resources/testData/SampleDataFile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frede\IdeaProjects\java\ExcelDataReader\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FEC463D-2F35-4BFA-851C-0D6AA8DB937B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE0918FB-6310-48AF-84FD-C24CB599AFED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -330,12 +330,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -363,6 +357,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -652,7 +652,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -670,13 +670,13 @@
       <c r="F1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="18"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -806,7 +806,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -844,7 +844,7 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A2" s="20"/>
+      <c r="A2" s="18"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" s="11" t="s">
@@ -975,7 +975,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1014,129 +1014,129 @@
       <c r="M1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="18" t="s">
+      <c r="N1" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
-      <c r="S1" s="18"/>
-      <c r="T1" s="18"/>
-      <c r="U1" s="18"/>
-      <c r="V1" s="18"/>
-      <c r="W1" s="18"/>
-      <c r="X1" s="18"/>
-      <c r="Y1" s="21" t="s">
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
+      <c r="T1" s="16"/>
+      <c r="U1" s="16"/>
+      <c r="V1" s="16"/>
+      <c r="W1" s="16"/>
+      <c r="X1" s="16"/>
+      <c r="Y1" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="Z1" s="22"/>
-      <c r="AA1" s="22"/>
-      <c r="AB1" s="22"/>
-      <c r="AC1" s="22"/>
-      <c r="AD1" s="22"/>
-      <c r="AE1" s="22"/>
-      <c r="AF1" s="22"/>
-      <c r="AG1" s="22"/>
-      <c r="AH1" s="22"/>
-      <c r="AI1" s="23"/>
+      <c r="Z1" s="20"/>
+      <c r="AA1" s="20"/>
+      <c r="AB1" s="20"/>
+      <c r="AC1" s="20"/>
+      <c r="AD1" s="20"/>
+      <c r="AE1" s="20"/>
+      <c r="AF1" s="20"/>
+      <c r="AG1" s="20"/>
+      <c r="AH1" s="20"/>
+      <c r="AI1" s="21"/>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A2" s="24"/>
-      <c r="N2" s="12" t="s">
+      <c r="A2" s="22"/>
+      <c r="N2" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="P2" s="12" t="s">
+      <c r="P2" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="Q2" s="12" t="s">
+      <c r="Q2" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="12" t="s">
+      <c r="R2" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="S2" s="12" t="s">
+      <c r="S2" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="T2" s="12" t="s">
+      <c r="T2" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="U2" s="12" t="s">
+      <c r="U2" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="V2" s="12" t="s">
+      <c r="V2" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="W2" s="12" t="s">
+      <c r="W2" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="X2" s="12" t="s">
+      <c r="X2" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="Y2" s="13" t="s">
+      <c r="Y2" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="Z2" s="13" t="s">
+      <c r="Z2" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="AA2" s="13" t="s">
+      <c r="AA2" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="AB2" s="13" t="s">
+      <c r="AB2" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="AC2" s="13" t="s">
+      <c r="AC2" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="AD2" s="13" t="s">
+      <c r="AD2" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="AE2" s="13" t="s">
+      <c r="AE2" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="AF2" s="13" t="s">
+      <c r="AF2" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="AG2" s="13" t="s">
+      <c r="AG2" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="AH2" s="13" t="s">
+      <c r="AH2" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="AI2" s="13" t="s">
+      <c r="AI2" s="25" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A3" s="25"/>
+      <c r="A3" s="23"/>
       <c r="B3" t="s">
         <v>35</v>
       </c>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
-      <c r="V3" s="12"/>
-      <c r="W3" s="12"/>
-      <c r="X3" s="12"/>
-      <c r="Y3" s="13"/>
-      <c r="Z3" s="13"/>
-      <c r="AA3" s="13"/>
-      <c r="AB3" s="13"/>
-      <c r="AC3" s="13"/>
-      <c r="AD3" s="13"/>
-      <c r="AE3" s="13"/>
-      <c r="AF3" s="13"/>
-      <c r="AG3" s="13"/>
-      <c r="AH3" s="13"/>
-      <c r="AI3" s="13"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="24"/>
+      <c r="R3" s="24"/>
+      <c r="S3" s="24"/>
+      <c r="T3" s="24"/>
+      <c r="U3" s="24"/>
+      <c r="V3" s="24"/>
+      <c r="W3" s="24"/>
+      <c r="X3" s="24"/>
+      <c r="Y3" s="24"/>
+      <c r="Z3" s="24"/>
+      <c r="AA3" s="24"/>
+      <c r="AB3" s="24"/>
+      <c r="AC3" s="24"/>
+      <c r="AD3" s="24"/>
+      <c r="AE3" s="24"/>
+      <c r="AF3" s="24"/>
+      <c r="AG3" s="24"/>
+      <c r="AH3" s="24"/>
+      <c r="AI3" s="24"/>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
@@ -1284,52 +1284,52 @@
       </c>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="Y6" s="14">
-        <v>123.56</v>
-      </c>
-      <c r="Z6" s="14" t="s">
+      <c r="Y6" s="12">
+        <v>123.56</v>
+      </c>
+      <c r="Z6" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="AA6" s="15">
-        <v>45424</v>
-      </c>
-      <c r="AB6" s="14">
-        <v>123.56</v>
-      </c>
-      <c r="AC6" s="14">
+      <c r="AA6" s="13">
+        <v>45424</v>
+      </c>
+      <c r="AB6" s="12">
+        <v>123.56</v>
+      </c>
+      <c r="AC6" s="12">
         <v>123</v>
       </c>
-      <c r="AD6" s="16">
+      <c r="AD6" s="14">
         <v>45424.548738425925</v>
       </c>
-      <c r="AE6" s="15">
-        <v>45424</v>
-      </c>
-      <c r="AF6" s="17">
+      <c r="AE6" s="13">
+        <v>45424</v>
+      </c>
+      <c r="AF6" s="15">
         <v>0.54873842592592592</v>
       </c>
-      <c r="AG6" s="14">
+      <c r="AG6" s="12">
         <v>123000</v>
       </c>
-      <c r="AH6" s="14" t="s">
+      <c r="AH6" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="AI6" s="14" t="s">
+      <c r="AI6" s="12" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="Y7" s="14"/>
-      <c r="Z7" s="14"/>
-      <c r="AA7" s="15"/>
-      <c r="AB7" s="14"/>
-      <c r="AC7" s="14"/>
-      <c r="AD7" s="16"/>
-      <c r="AE7" s="15"/>
-      <c r="AF7" s="17"/>
-      <c r="AG7" s="14"/>
-      <c r="AH7" s="14"/>
-      <c r="AI7" s="14"/>
+      <c r="Y7" s="12"/>
+      <c r="Z7" s="12"/>
+      <c r="AA7" s="13"/>
+      <c r="AB7" s="12"/>
+      <c r="AC7" s="12"/>
+      <c r="AD7" s="14"/>
+      <c r="AE7" s="13"/>
+      <c r="AF7" s="15"/>
+      <c r="AG7" s="12"/>
+      <c r="AH7" s="12"/>
+      <c r="AI7" s="12"/>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">

</xml_diff>

<commit_message>
Added the capability to get test data from a reference
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/SampleDataFile.xlsx
+++ b/src/test/resources/testData/SampleDataFile.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frede\IdeaProjects\java\ExcelDataReader\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE0918FB-6310-48AF-84FD-C24CB599AFED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86522977-AF22-442A-BB47-B7B00BE51130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SampleDataRecord" sheetId="1" r:id="rId1"/>
@@ -334,6 +334,12 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -357,12 +363,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -652,7 +652,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -670,13 +670,13 @@
       <c r="F1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="16"/>
+      <c r="H1" s="18"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A2" s="17"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -806,7 +806,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -844,7 +844,7 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A2" s="18"/>
+      <c r="A2" s="20"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" s="11" t="s">
@@ -975,7 +975,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1014,129 +1014,129 @@
       <c r="M1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="N1" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="T1" s="16"/>
-      <c r="U1" s="16"/>
-      <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
-      <c r="X1" s="16"/>
-      <c r="Y1" s="19" t="s">
+      <c r="O1" s="18"/>
+      <c r="P1" s="18"/>
+      <c r="Q1" s="18"/>
+      <c r="R1" s="18"/>
+      <c r="S1" s="18"/>
+      <c r="T1" s="18"/>
+      <c r="U1" s="18"/>
+      <c r="V1" s="18"/>
+      <c r="W1" s="18"/>
+      <c r="X1" s="18"/>
+      <c r="Y1" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="Z1" s="20"/>
-      <c r="AA1" s="20"/>
-      <c r="AB1" s="20"/>
-      <c r="AC1" s="20"/>
-      <c r="AD1" s="20"/>
-      <c r="AE1" s="20"/>
-      <c r="AF1" s="20"/>
-      <c r="AG1" s="20"/>
-      <c r="AH1" s="20"/>
-      <c r="AI1" s="21"/>
+      <c r="Z1" s="22"/>
+      <c r="AA1" s="22"/>
+      <c r="AB1" s="22"/>
+      <c r="AC1" s="22"/>
+      <c r="AD1" s="22"/>
+      <c r="AE1" s="22"/>
+      <c r="AF1" s="22"/>
+      <c r="AG1" s="22"/>
+      <c r="AH1" s="22"/>
+      <c r="AI1" s="23"/>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A2" s="22"/>
-      <c r="N2" s="25" t="s">
+      <c r="A2" s="24"/>
+      <c r="N2" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="O2" s="25" t="s">
+      <c r="O2" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="P2" s="25" t="s">
+      <c r="P2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="Q2" s="25" t="s">
+      <c r="Q2" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="25" t="s">
+      <c r="R2" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="S2" s="25" t="s">
+      <c r="S2" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="T2" s="25" t="s">
+      <c r="T2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="U2" s="25" t="s">
+      <c r="U2" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="V2" s="25" t="s">
+      <c r="V2" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="W2" s="25" t="s">
+      <c r="W2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="X2" s="25" t="s">
+      <c r="X2" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="Y2" s="25" t="s">
+      <c r="Y2" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="Z2" s="25" t="s">
+      <c r="Z2" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="AA2" s="25" t="s">
+      <c r="AA2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="AB2" s="25" t="s">
+      <c r="AB2" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="AC2" s="25" t="s">
+      <c r="AC2" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="AD2" s="25" t="s">
+      <c r="AD2" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="AE2" s="25" t="s">
+      <c r="AE2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="AF2" s="25" t="s">
+      <c r="AF2" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="AG2" s="25" t="s">
+      <c r="AG2" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="AH2" s="25" t="s">
+      <c r="AH2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="AI2" s="25" t="s">
+      <c r="AI2" s="17" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.45">
-      <c r="A3" s="23"/>
+      <c r="A3" s="25"/>
       <c r="B3" t="s">
         <v>35</v>
       </c>
-      <c r="N3" s="24"/>
-      <c r="O3" s="24"/>
-      <c r="P3" s="24"/>
-      <c r="Q3" s="24"/>
-      <c r="R3" s="24"/>
-      <c r="S3" s="24"/>
-      <c r="T3" s="24"/>
-      <c r="U3" s="24"/>
-      <c r="V3" s="24"/>
-      <c r="W3" s="24"/>
-      <c r="X3" s="24"/>
-      <c r="Y3" s="24"/>
-      <c r="Z3" s="24"/>
-      <c r="AA3" s="24"/>
-      <c r="AB3" s="24"/>
-      <c r="AC3" s="24"/>
-      <c r="AD3" s="24"/>
-      <c r="AE3" s="24"/>
-      <c r="AF3" s="24"/>
-      <c r="AG3" s="24"/>
-      <c r="AH3" s="24"/>
-      <c r="AI3" s="24"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="16"/>
+      <c r="S3" s="16"/>
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
+      <c r="V3" s="16"/>
+      <c r="W3" s="16"/>
+      <c r="X3" s="16"/>
+      <c r="Y3" s="16"/>
+      <c r="Z3" s="16"/>
+      <c r="AA3" s="16"/>
+      <c r="AB3" s="16"/>
+      <c r="AC3" s="16"/>
+      <c r="AD3" s="16"/>
+      <c r="AE3" s="16"/>
+      <c r="AF3" s="16"/>
+      <c r="AG3" s="16"/>
+      <c r="AH3" s="16"/>
+      <c r="AI3" s="16"/>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
@@ -1341,7 +1341,7 @@
       <c r="C8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="9">
         <v>45424</v>
       </c>
       <c r="E8" s="2">
@@ -1350,13 +1350,13 @@
       <c r="F8" s="2">
         <v>123</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="8">
         <v>45424.548738425925</v>
       </c>
-      <c r="H8" s="2">
-        <v>45424</v>
-      </c>
-      <c r="I8" s="2">
+      <c r="H8" s="9">
+        <v>45424</v>
+      </c>
+      <c r="I8" s="10">
         <v>0.54873842592592592</v>
       </c>
       <c r="J8" s="2">
@@ -1377,7 +1377,7 @@
       <c r="O8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="9">
         <v>45424</v>
       </c>
       <c r="Q8" s="2">
@@ -1386,13 +1386,13 @@
       <c r="R8" s="2">
         <v>123</v>
       </c>
-      <c r="S8" s="2">
+      <c r="S8" s="8">
         <v>45424.548738425925</v>
       </c>
-      <c r="T8" s="2">
-        <v>45424</v>
-      </c>
-      <c r="U8" s="2">
+      <c r="T8" s="9">
+        <v>45424</v>
+      </c>
+      <c r="U8" s="10">
         <v>0.54873842592592592</v>
       </c>
       <c r="V8" s="2">
@@ -1410,7 +1410,7 @@
       <c r="Z8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="AA8" s="2">
+      <c r="AA8" s="9">
         <v>45424</v>
       </c>
       <c r="AB8" s="2">
@@ -1419,13 +1419,13 @@
       <c r="AC8" s="2">
         <v>123</v>
       </c>
-      <c r="AD8" s="2">
+      <c r="AD8" s="8">
         <v>45424.548738425925</v>
       </c>
-      <c r="AE8" s="2">
-        <v>45424</v>
-      </c>
-      <c r="AF8" s="2">
+      <c r="AE8" s="9">
+        <v>45424</v>
+      </c>
+      <c r="AF8" s="10">
         <v>0.54873842592592592</v>
       </c>
       <c r="AG8" s="2">
@@ -1471,7 +1471,7 @@
       <c r="Z9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="AA9" s="2">
+      <c r="AA9" s="9">
         <v>45424</v>
       </c>
       <c r="AB9" s="2">
@@ -1480,13 +1480,13 @@
       <c r="AC9" s="2">
         <v>123</v>
       </c>
-      <c r="AD9" s="2">
+      <c r="AD9" s="8">
         <v>45424.548738425925</v>
       </c>
-      <c r="AE9" s="2">
-        <v>45424</v>
-      </c>
-      <c r="AF9" s="2">
+      <c r="AE9" s="9">
+        <v>45424</v>
+      </c>
+      <c r="AF9" s="10">
         <v>0.54873842592592592</v>
       </c>
       <c r="AG9" s="2">
@@ -1506,7 +1506,7 @@
       <c r="Z10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="AA10" s="2">
+      <c r="AA10" s="9">
         <v>45424</v>
       </c>
       <c r="AB10" s="2">
@@ -1515,13 +1515,13 @@
       <c r="AC10" s="2">
         <v>123</v>
       </c>
-      <c r="AD10" s="2">
+      <c r="AD10" s="8">
         <v>45424.548738425925</v>
       </c>
-      <c r="AE10" s="2">
-        <v>45424</v>
-      </c>
-      <c r="AF10" s="2">
+      <c r="AE10" s="9">
+        <v>45424</v>
+      </c>
+      <c r="AF10" s="10">
         <v>0.54873842592592592</v>
       </c>
       <c r="AG10" s="2">

</xml_diff>